<commit_message>
updated the testCases excel file
</commit_message>
<xml_diff>
--- a/IMDB Test Cases.xlsx
+++ b/IMDB Test Cases.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30203"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="151" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46E954E6-A0ED-4AF2-B92A-6B3BE7D9AC20}"/>
+  <xr:revisionPtr revIDLastSave="163" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{096BB01A-E72E-47B4-8EFD-BADBA1E0B622}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="60">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -83,6 +83,15 @@
     <t>The searched movie page load with the correct movie title.</t>
   </si>
   <si>
+    <t>As Expected</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
     <t>WF1-02</t>
   </si>
   <si>
@@ -137,7 +146,7 @@
     <t>WF1-05</t>
   </si>
   <si>
-    <t>Searching for a non-existant movie</t>
+    <t>Searching for a non-existent movie</t>
   </si>
   <si>
     <t>Movie Title: xyzqwe123456789</t>
@@ -187,7 +196,7 @@
   <si>
     <t>1. Click the Sort by button.
 2. Select (Alphabetical).
-3. Check the names of the first 3 movies titles.</t>
+3. Check the names of the first 10 movies titles.</t>
   </si>
   <si>
     <t>The table updates smoothly and the top movies are sorted alphabeticaly.</t>
@@ -216,6 +225,9 @@
     <t>1. Store the exact title text string of the movie in row #5.
 2. Click directly on that movie's title link.
 3. Check the title from the new page view.</t>
+  </si>
+  <si>
+    <t>The browser successfullygoes to the clicked movie titles page and shows the desired movie information.</t>
   </si>
 </sst>
 </file>
@@ -252,7 +264,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -367,21 +379,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -401,21 +398,6 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
@@ -430,7 +412,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -456,23 +438,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -849,204 +828,266 @@
       <c r="F2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="9"/>
+      <c r="G2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="91.5">
-      <c r="A3" s="10" t="s">
-        <v>15</v>
+      <c r="A3" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="11"/>
     </row>
     <row r="4" spans="1:9" ht="121.5">
-      <c r="A4" s="10" t="s">
-        <v>20</v>
+      <c r="A4" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="11"/>
+        <v>27</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" spans="1:9" ht="76.5">
-      <c r="A5" s="10" t="s">
-        <v>25</v>
+      <c r="A5" s="9" t="s">
+        <v>28</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="11"/>
+        <v>33</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="106.5">
-      <c r="A6" s="10" t="s">
-        <v>31</v>
+      <c r="A6" s="9" t="s">
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="11"/>
+        <v>38</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:9" ht="106.5">
-      <c r="A7" s="10" t="s">
-        <v>36</v>
+      <c r="A7" s="9" t="s">
+        <v>39</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="11"/>
+        <v>42</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="91.5">
-      <c r="A8" s="10" t="s">
-        <v>40</v>
+      <c r="A8" s="9" t="s">
+        <v>43</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="11"/>
+        <v>46</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="76.5">
-      <c r="A9" s="10" t="s">
-        <v>44</v>
+      <c r="A9" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="11"/>
+        <v>51</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="106.5">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="11"/>
+        <v>55</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="106.5">
-      <c r="A11" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>54</v>
+      <c r="A11" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>57</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="14"/>
+        <v>49</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>